<commit_message>
Document profile, pending-account, and rejection tests; retest fixes and remaining failures
</commit_message>
<xml_diff>
--- a/docs/tests/GoGallery_Failed_Tests.xlsx
+++ b/docs/tests/GoGallery_Failed_Tests.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="160">
   <si>
     <t>No.</t>
   </si>
@@ -373,6 +373,44 @@
     <t>docs/tests/portal-utama/evidence/ptu-home-final.png</t>
   </si>
   <si>
+    <t>Unapproved accounts</t>
+  </si>
+  <si>
+    <t>PND-08</t>
+  </si>
+  <si>
+    <t>Unapproved Galeri listed in the public directory</t>
+  </si>
+  <si>
+    <t>Unapproved account visible publicly</t>
+  </si>
+  <si>
+    <t>Galeri (unapproved)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Use a Galeri account that admin has not approved (still in Barisan semakan).
+2. Upload a profile photo in Profil Saya.
+3. As an anonymous visitor open /resources/galleries?search=&lt;name&gt; and the profile page.</t>
+  </si>
+  <si>
+    <t>Not listed until admin approves the membership (an unapproved Artist is hidden; registration says profiles show after admin review).</t>
+  </si>
+  <si>
+    <t>The Galeri is listed (Galeri 0) with its uploaded photo and its profile page opens (200). The pending Artist is not listed.</t>
+  </si>
+  <si>
+    <t>Anyone can appear in the public gallery directory with a name and photo without admin review.</t>
+  </si>
+  <si>
+    <t>Defect. Also decide whether unapproved accounts may upload at all (pending-accounts/FAILURES.md N-I1).</t>
+  </si>
+  <si>
+    <t>docs/tests/pending-accounts/PND-08-galeri-public-before-approval.md</t>
+  </si>
+  <si>
+    <t>docs/tests/pending-accounts/evidence/public-galeri-dir.png</t>
+  </si>
+  <si>
     <t>Test</t>
   </si>
   <si>
@@ -458,6 +496,9 @@
   </si>
   <si>
     <t>Add server-side URL validation like the Berita link field (require http/https; reject javascript: and spaces).</t>
+  </si>
+  <si>
+    <t>Hide unapproved Galeri accounts from the public directory and profile pages like Artists; decide whether unapproved accounts may upload at all.</t>
   </si>
   <si>
     <t>Add the same confirmation dialog used by other modules to banner delete.</t>
@@ -907,7 +948,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:T10"/>
+  <dimension ref="A1:T11"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -1548,19 +1589,81 @@
         <v>36</v>
       </c>
     </row>
+    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A11" s="2">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="I11" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="J11" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="K11" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="L11" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="M11" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="N11" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="O11" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="P11" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q11" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="R11" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="S11" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="T11" s="2" t="s">
+        <v>36</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:T1"/>
   <dataValidations count="4">
-    <dataValidation type="list" allowBlank="1" sqref="Q10">
+    <dataValidation type="list" allowBlank="1" sqref="Q10:Q11">
       <formula1>"Open,In progress,Fixed,Won't fix,Needs decision"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="Q2:Q10">
+    <dataValidation type="list" allowBlank="1" sqref="Q2:Q11">
       <formula1>"Open,In progress,Fixed,Won't fix,Needs decision"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="S10">
+    <dataValidation type="list" allowBlank="1" sqref="S10:S11">
       <formula1>"Pass,Fail,Not retested"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="S2:S10">
+    <dataValidation type="list" allowBlank="1" sqref="S2:S11">
       <formula1>"Pass,Fail,Not retested"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1594,16 +1697,16 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>114</v>
+        <v>126</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>7</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>115</v>
+        <v>127</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>116</v>
+        <v>128</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>13</v>
@@ -1617,22 +1720,22 @@
         <v>63</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>117</v>
+        <v>129</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>118</v>
+        <v>130</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>119</v>
+        <v>131</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>120</v>
+        <v>132</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>121</v>
+        <v>133</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>122</v>
+        <v>134</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1640,25 +1743,25 @@
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>123</v>
+        <v>135</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>124</v>
+        <v>136</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>126</v>
+        <v>138</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>127</v>
+        <v>139</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>128</v>
+        <v>140</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>129</v>
+        <v>141</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -1666,25 +1769,25 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>118</v>
-      </c>
       <c r="E4" s="2" t="s">
-        <v>126</v>
+        <v>138</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>127</v>
+        <v>139</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>132</v>
+        <v>144</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>133</v>
+        <v>145</v>
       </c>
     </row>
   </sheetData>
@@ -1696,7 +1799,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -1711,16 +1814,16 @@
         <v>6</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>134</v>
+        <v>146</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>135</v>
+        <v>147</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>136</v>
+        <v>148</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>137</v>
+        <v>149</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -1728,7 +1831,7 @@
         <v>25</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>138</v>
+        <v>150</v>
       </c>
       <c r="C2" s="2">
         <v>5</v>
@@ -1737,7 +1840,7 @@
         <v>24</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>139</v>
+        <v>151</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
@@ -1754,7 +1857,7 @@
         <v>24</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>140</v>
+        <v>152</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -1762,7 +1865,7 @@
         <v>87</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>141</v>
+        <v>153</v>
       </c>
       <c r="C4" s="2">
         <v>2</v>
@@ -1771,15 +1874,15 @@
         <v>86</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>142</v>
+        <v>154</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>106</v>
+        <v>117</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>104</v>
+        <v>115</v>
       </c>
       <c r="C5" s="2">
         <v>1</v>
@@ -1788,28 +1891,45 @@
         <v>86</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="6" t="s">
-        <v>144</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="C7" s="6">
-        <v>9</v>
+        <v>155</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="C6" s="2">
+        <v>1</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>156</v>
       </c>
     </row>
     <row r="8" spans="1:3" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
-        <v>145</v>
+        <v>157</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>146</v>
+        <v>36</v>
       </c>
       <c r="C8" s="6">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="6" t="s">
+        <v>158</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="C9" s="6">
         <v>3</v>
       </c>
     </row>

</xml_diff>